<commit_message>
adding more SP title and locaiton validations mainly for transfers
</commit_message>
<xml_diff>
--- a/tests/TeamworkDB/output/utilization_failures_report_202608.xlsx
+++ b/tests/TeamworkDB/output/utilization_failures_report_202608.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Employee Monthly" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Employee YTD" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terminated Employee Visibility" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster Completeness" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1395,17 +1396,17 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>3,970.70</t>
+          <t>3,979.00</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>157.10</t>
+          <t>165.40</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>4.12%</t>
+          <t>4.34%</t>
         </is>
       </c>
     </row>
@@ -1617,17 +1618,17 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>2,807,747.00</t>
+          <t>2,813,349.00</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>120,182.00</t>
+          <t>125,784.00</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>4.47%</t>
+          <t>4.68%</t>
         </is>
       </c>
     </row>
@@ -3253,17 +3254,17 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>34,575.10</t>
+          <t>34,583.40</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>5,346.35</t>
+          <t>5,354.65</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>18.29%</t>
+          <t>18.32%</t>
         </is>
       </c>
     </row>
@@ -3549,17 +3550,17 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>34,458.30</t>
+          <t>34,461.30</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>8,151.66</t>
+          <t>8,154.66</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>30.99%</t>
+          <t>31.00%</t>
         </is>
       </c>
     </row>
@@ -3808,17 +3809,17 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>8,803.00</t>
+          <t>8,807.60</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>1,826.30</t>
+          <t>1,821.70</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>17.18%</t>
+          <t>17.14%</t>
         </is>
       </c>
     </row>
@@ -3956,17 +3957,17 @@
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>25,582,200.00</t>
+          <t>25,587,803.00</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>4,772,110.25</t>
+          <t>4,777,713.25</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>22.93%</t>
+          <t>22.96%</t>
         </is>
       </c>
     </row>
@@ -4252,17 +4253,17 @@
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>26,295,409.00</t>
+          <t>26,297,704.00</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>7,006,880.40</t>
+          <t>7,009,175.40</t>
         </is>
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>
-          <t>36.33%</t>
+          <t>36.34%</t>
         </is>
       </c>
     </row>
@@ -4511,17 +4512,17 @@
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>8,417,517.00</t>
+          <t>8,421,772.00</t>
         </is>
       </c>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>1,570,617.50</t>
+          <t>1,566,362.50</t>
         </is>
       </c>
       <c r="G104" s="4" t="inlineStr">
         <is>
-          <t>15.72%</t>
+          <t>15.68%</t>
         </is>
       </c>
     </row>
@@ -5062,7 +5063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5470,267 +5471,267 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>101279</t>
+          <t>102296</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Lee, Shinyoung</t>
+          <t>Han, Yvonne</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Standard_Rev</t>
+          <t>Actual_Hours</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>134,131.50</t>
+          <t>167.40</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>143,603.00</t>
+          <t>175.70</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>9,471.50</t>
+          <t>8.30</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>7.06%</t>
+          <t>4.96%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>101279</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Lee, Shinyoung</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>134,131.50</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>143,603.00</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>9,471.50</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>7.06%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>101644</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Murphy, Kevin</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Standard_Rev</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>62,215.00</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>67,620.00</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>5,405.00</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>8.69%</t>
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>102296</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Han, Yvonne</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>112,995.00</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>118,598.00</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>5,603.00</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>4.96%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Sheet: Month - CRDC (Monthly)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Util Report</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>DB</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Diff</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Diff%</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>101387</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Foley, Conor</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Target_Hours</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>155.40</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>146.30</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>9.10</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>5.86%</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>101387</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Foley, Conor</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Target_Rev</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>143,745.00</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>135,360.00</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>8,385.00</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>5.83%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>101528</t>
+          <t>101387</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Podwol, Joseph</t>
+          <t>Foley, Conor</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Actual_Hours</t>
+          <t>Target_Hours</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>33.40</t>
+          <t>155.40</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>58.70</t>
+          <t>146.30</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>25.30</t>
+          <t>9.10</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>75.75%</t>
+          <t>5.86%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>101591</t>
+          <t>101387</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Jones, Nate</t>
+          <t>Foley, Conor</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Actual_Hours</t>
+          <t>Target_Rev</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>111.80</t>
+          <t>143,745.00</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>117.80</t>
+          <t>135,360.00</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>6.00</t>
+          <t>8,385.00</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>5.37%</t>
+          <t>5.83%</t>
         </is>
       </c>
     </row>
@@ -5747,22 +5748,22 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Standard_Rev</t>
+          <t>Actual_Hours</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>37,575.00</t>
+          <t>33.40</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>66,038.00</t>
+          <t>58.70</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>28,463.00</t>
+          <t>25.30</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -5784,146 +5785,146 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>111.80</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>117.80</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>6.00</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>5.37%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>101528</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Podwol, Joseph</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
           <t>Standard_Rev</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>37,575.00</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>66,038.00</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>28,463.00</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>75.75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>101591</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Jones, Nate</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>54,223.00</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>57,133.00</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>2,910.00</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>5.37%</t>
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Sheet: Month - CRNY (Monthly)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Util Report</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>DB</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Diff</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Diff%</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>102079</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Solaeche, Guadalupe</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Actual_Hours</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>50.30</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>53.20</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>2.90</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>5.77%</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>102219</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Shah, Shriya</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Actual_Hours</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>119.40</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>128.50</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>9.10</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>7.62%</t>
         </is>
       </c>
     </row>
@@ -5940,22 +5941,22 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Standard_Rev</t>
+          <t>Actual_Hours</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>21,880.50</t>
+          <t>50.30</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>23,142.00</t>
+          <t>53.20</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>1,261.50</t>
+          <t>2.90</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -5977,277 +5978,277 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>119.40</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>128.50</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>9.10</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>7.62%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>102079</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Solaeche, Guadalupe</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
           <t>Standard_Rev</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>21,880.50</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>23,142.00</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>1,261.50</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>5.77%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>102219</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Shah, Shriya</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>51,939.00</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>55,898.00</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>3,959.00</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>7.62%</t>
         </is>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Sheet: Month - CRSV (Monthly)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>Util Report</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>DB</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>Diff</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Diff%</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>101961</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Jang, Ryan</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Actual_Hours</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>114.60</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>123.00</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>8.40</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>7.33%</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>101961</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Jang, Ryan</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Standard_Rev</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>55,581.00</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>59,655.00</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>4,074.00</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>7.33%</t>
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Sheet: Month - CRUK (Monthly)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>Util Report</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>DB</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Diff</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Diff%</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>0543</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Bredendiek, Maximilian</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Actual_Hours</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>112.90</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>118.50</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>5.60</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>4.96%</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>101964</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Roketskiy, Nikita</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Actual_Hours</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>90.80</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>98.00</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>7.20</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>7.93%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>102337</t>
+          <t>0543</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Williams, Ryan</t>
+          <t>Bredendiek, Maximilian</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -6257,22 +6258,22 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>147.50</t>
+          <t>112.90</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>158.50</t>
+          <t>118.50</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>11.00</t>
+          <t>5.60</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>7.46%</t>
+          <t>4.96%</t>
         </is>
       </c>
     </row>
@@ -6289,22 +6290,22 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Standard_Rev</t>
+          <t>Actual_Hours</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>76,516.02</t>
+          <t>90.80</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>82,583.00</t>
+          <t>98.00</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>6,066.98</t>
+          <t>7.20</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -6326,35 +6327,101 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
+          <t>Actual_Hours</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>147.50</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>158.50</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>11.00</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>7.46%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>101964</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Roketskiy, Nikita</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
           <t>Standard_Rev</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>76,516.02</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>82,583.00</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>6,066.98</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>7.93%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>102337</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Williams, Ryan</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>176,003.71</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>189,129.00</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>13,125.29</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>7.46%</t>
-        </is>
-      </c>
-    </row>
-    <row r="47"/>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>MISSING ROWS</t>
         </is>
       </c>
     </row>
@@ -6362,399 +6429,353 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
+          <t>MISSING ROWS</t>
+        </is>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
           <t>Sheet: Month - CRB  (Monthly)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>Name</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>MISSING IN DB</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>101372</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>Lobo, Isabelle</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Employee_name: Lobo, Isabelle</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>OFFC: CRNY</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>Total_Billable_Hours: 111.3000</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>MISSING IN DB</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>102071</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>Hsu, Caroline</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Employee_name: Hsu, Caroline</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>OFFC: CRNY</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
-        <is>
-          <t>Total_Billable_Hours: 68.6000</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
+          <t>MISSING IN DB</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>101372</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Lobo, Isabelle</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Employee_name: Lobo, Isabelle</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>OFFC: CRNY</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Total_Billable_Hours: 111.3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>MISSING IN DB</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>102071</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Hsu, Caroline</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Employee_name: Hsu, Caroline</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>OFFC: CRNY</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Total_Billable_Hours: 68.6000</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
           <t>MISSING IN XLS</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>101409</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>Target_Hrs: 148.00000000000006</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>Actual_Hrs: 197.19999999999996</t>
         </is>
       </c>
     </row>
-    <row r="55"/>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+    <row r="57"/>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Sheet: Month - CRCH (Monthly)</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>MISSING IN XLS</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>101102</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>Target_Hrs: 160.0</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>Actual_Hrs: 157.10000000000002</t>
         </is>
       </c>
     </row>
-    <row r="59"/>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+    <row r="61"/>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>Sheet: Month - CRDC (Monthly)</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>MISSING IN DB</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>102067</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>Gould, Naomi</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>Employee_name: Gould, Naomi</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>OFFC: CRNY</t>
         </is>
       </c>
-      <c r="F62" s="5" t="inlineStr">
+      <c r="F64" s="5" t="inlineStr">
         <is>
           <t>Total_Billable_Hours: 23.0000</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>MISSING IN DB</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>102077</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>Hagerty, Matthew</t>
         </is>
       </c>
-      <c r="D63" s="5" t="inlineStr">
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t>Employee_name: Hagerty, Matthew</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>OFFC: CRNY</t>
         </is>
       </c>
-      <c r="F63" s="5" t="inlineStr">
+      <c r="F65" s="5" t="inlineStr">
         <is>
           <t>Total_Billable_Hours: 100.8000</t>
         </is>
       </c>
     </row>
-    <row r="64"/>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+    <row r="66"/>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>Sheet: Month - CRNY (Monthly)</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>Name</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>MISSING IN DB</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>101102</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>Nandwani, Gehna Rai</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Employee_name: Nandwani, Gehna Rai</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>OFFC: CRCH</t>
-        </is>
-      </c>
-      <c r="F67" s="5" t="inlineStr">
-        <is>
-          <t>Total_Billable_Hours: 157.1000</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>MISSING IN DB</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>101409</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Trubnikova, Anna</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Employee_name: Trubnikova, Anna</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>OFFC: CRB</t>
-        </is>
-      </c>
-      <c r="F68" s="5" t="inlineStr">
-        <is>
-          <t>Total_Billable_Hours: 197.2000</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>MISSING IN XLS</t>
+          <t>MISSING IN DB</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>101372</t>
+          <t>101102</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Nandwani, Gehna Rai</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Target_Hrs: 160.0</t>
+          <t>Employee_name: Nandwani, Gehna Rai</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>Actual_Hrs: 111.29999999999998</t>
+          <t>OFFC: CRCH</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Total_Billable_Hours: 157.1000</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>MISSING IN XLS</t>
+          <t>MISSING IN DB</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>102067</t>
+          <t>101409</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Trubnikova, Anna</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Target_Hrs: 120.0</t>
+          <t>Employee_name: Trubnikova, Anna</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Actual_Hrs: 23.0</t>
+          <t>OFFC: CRB</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Total_Billable_Hours: 197.2000</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6787,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>102071</t>
+          <t>101372</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -6776,12 +6797,12 @@
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>Target_Hrs: 168.0</t>
+          <t>Target_Hrs: 160.0</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>Actual_Hrs: 68.6</t>
+          <t>Actual_Hrs: 111.29999999999998</t>
         </is>
       </c>
     </row>
@@ -6793,20 +6814,74 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
+          <t>102067</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Target_Hrs: 120.0</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Actual_Hrs: 23.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>MISSING IN XLS</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>102071</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Target_Hrs: 168.0</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Actual_Hrs: 68.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>MISSING IN XLS</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
           <t>102077</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="D72" s="5" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>Target_Hrs: 168.0</t>
         </is>
       </c>
-      <c r="E72" s="5" t="inlineStr">
+      <c r="E74" s="5" t="inlineStr">
         <is>
           <t>Actual_Hrs: 100.8</t>
         </is>
@@ -60232,4 +60307,345 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Roster Completeness</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>FORMAT ERRORS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sheet: </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>MISSING FROM MONTHLY REPORT</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5905 | Name=Christina Zafeiridou | Office=London | Dept=1000 | Status=Active | HireDate=2025-08-03 | TermDate=Active | Level=P3UK | JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MISSING FROM YTD REPORT</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5905 | Name=Christina Zafeiridou | Office=London | Dept=1000 | Status=Active | HireDate=2025-08-03 | TermDate=Active | Level=P3UK | JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5369 | Name=Vijeta Graham | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5483 | Name=Etienne Cayer | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5624 | Name=Prithvi Hingorani | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5766 | Name=Austin Schwed | Expected_Title=Manager | Actual_SP_Title=SRA/Associate | Actual_Group=Associate | Workday_Level=M1 | Workday_JobTitle=Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5802 | Name=Burkett Evans | Expected_Title=Manager | Actual_SP_Title=SRA/Associate | Actual_Group=Associate | Workday_Level=M1 | Workday_JobTitle=Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5967 | Name=Spencer Vernon | Expected_Title=Manager | Actual_SP_Title=SRA/Associate | Actual_Group=Associate | Workday_Level=M1 | Workday_JobTitle=Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6122 | Name=Michael Hilfiker | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6330 | Name=Alejandro Hoyos Suarez | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6333 | Name=Julia Russell | Expected_Title=Manager | Actual_SP_Title=SRA/Associate | Actual_Group=Associate | Workday_Level=M1 | Workday_JobTitle=Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6337 | Name=Benjamin Murphy | Expected_Title=Manager | Actual_SP_Title=SRA/Associate | Actual_Group=Associate | Workday_Level=M1 | Workday_JobTitle=Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6342 | Name=Samuel Haltenhof | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6354 | Name=Arthur Corea-Smith | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6383 | Name=Matthew Davis | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=0531 | Name=Hannah Tilson | Expected_Title=Manager | Actual_SP_Title=SRA/Associate | Actual_Group=Associate | Workday_Level=M1UK | Workday_JobTitle=Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=0543 | Name=Maximilian Bredendiek | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1UK | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=4876 | Name=Avishai Schiff | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6410 | Name=Molly Glandon | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6415 | Name=Chady Gemayel | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=6135 | Name=Kathleen Hu | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5100 | Name=Charles Boyer | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5432 | Name=Kathryn Fox | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>WRONG TITLE</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>EmpNo=5161 | Name=Bryan Pine | Expected_Title=Principal | Actual_SP_Title=Senior Manager | Actual_Group=Manager | Workday_Level=P1 | Workday_JobTitle=Principal</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>